<commit_message>
Rename AEDP to ACAP-EDP, restore aggregated datasets, withdraw single-household samples
- Rename every AEDP and Darth EDP reference to ACAP-EDP across paths,
  notebooks, scripts, result labels, docs and dataset metadata
- Restore the 18 aggregated ACAP-EDP datasets to data/ under the new names
  and register ds28-ds36 in the dataset download maps
- Remove the single-household samples ds25-ds27 from the published data
  folders and the aggregation batch spec
- Add the ACAP-EDP acknowledgement to the docs, README and metadata
- Regenerate the affected figures and tables so titles carry the new name

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$I$38</definedName>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,19 +562,16 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ds2_aedp_5min</t>
+          <t>ds2_acap-edp_5min</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia</t>
+          <t>ACAP-EDP dataset, aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -584,7 +581,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -612,12 +609,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ds3_aedp_30min</t>
+          <t>ds3_acap-edp_30min</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia</t>
+          <t>ACAP-EDP dataset, aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -627,7 +624,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -689,19 +686,16 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ds5_aedp_30min_with_weather</t>
+          <t>ds5_acap-edp_30min_with_weather</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia  plus weather data from BOM Sydney Airport data</t>
+          <t>ACAP-EDP dataset, aggregate of 487 households from Solar Analytics and Wattwatchers from all regions in Australia  plus weather data from BOM Sydney Airport data</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -711,7 +705,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -739,12 +733,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ds6_aedp_cluster_5min</t>
+          <t>ds6_acap-edp_cluster_5min</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -754,7 +748,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -782,12 +776,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ds7_aedp_cluster_30min</t>
+          <t>ds7_acap-edp_cluster_30min</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -797,7 +791,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -825,12 +819,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ds8_aedp_cluster_30min_with_weather</t>
+          <t>ds8_acap-edp_cluster_30min_with_weather</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 213 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -840,7 +834,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -868,12 +862,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ds9_aedp_cluster2_5min</t>
+          <t>ds9_acap-edp_cluster2_5min</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,7 +877,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -911,12 +905,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ds10_aedp_cluster2_30min</t>
+          <t>ds10_acap-edp_cluster2_30min</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -926,7 +920,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -954,12 +948,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ds11_aedp_cluster2_30min_with_weather</t>
+          <t>ds11_acap-edp_cluster2_30min_with_weather</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Australia Energy Data Platform Dataset, Aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
+          <t>ACAP-EDP dataset, aggregate of 148 households from Solar Analytics and Wattwatchers located in NSW</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -969,7 +963,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Solar Analytics, Wattwatchers collected in Darth</t>
+          <t>ACAP Energy Data Platform (Solar Analytics, Wattwatchers)</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -1389,7 +1383,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Uses Sydney Airport BOM station 066037 and the same weather variables as AEDP ds11.</t>
+          <t>Uses Sydney Airport BOM station 066037 and the same weather variables as ACAP-EDP ds11.</t>
         </is>
       </c>
     </row>
@@ -1580,12 +1574,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ds25_aedp_1hh_sample01_30min_with_weather</t>
+          <t>ds28_acap-edp_10hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 10 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1595,7 +1589,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
@@ -1616,19 +1610,19 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ds26_aedp_1hh_sample02_30min_with_weather</t>
+          <t>ds29_acap-edp_10hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 10 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1638,7 +1632,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
@@ -1659,19 +1653,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ds27_aedp_1hh_sample03_30min_with_weather</t>
+          <t>ds30_acap-edp_10hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 10 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1681,7 +1675,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
@@ -1702,19 +1696,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ds28_aedp_10hh_sample01_30min_with_weather</t>
+          <t>ds31_acap-edp_100hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 100 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1724,7 +1718,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
@@ -1745,19 +1739,19 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ds29_aedp_10hh_sample02_30min_with_weather</t>
+          <t>ds32_acap-edp_100hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 100 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1767,7 +1761,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
@@ -1788,19 +1782,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ds30_aedp_10hh_sample03_30min_with_weather</t>
+          <t>ds33_acap-edp_100hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, 100 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1810,7 +1804,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
@@ -1831,19 +1825,19 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ds31_aedp_100hh_sample01_30min_with_weather</t>
+          <t>ds34_acap-edp_1000hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1853,7 +1847,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
@@ -1874,19 +1868,19 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ds32_aedp_100hh_sample02_30min_with_weather</t>
+          <t>ds35_acap-edp_1000hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1896,7 +1890,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
@@ -1917,19 +1911,19 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ds33_aedp_100hh_sample03_30min_with_weather</t>
+          <t>ds36_acap-edp_1000hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+          <t>ACAP-EDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1939,7 +1933,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AEDP, BOM weather data</t>
+          <t>ACAP-EDP, BOM weather data</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
@@ -1960,136 +1954,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>ds34_aedp_1000hh_sample01_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 01, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>44378</v>
-      </c>
-      <c r="F36" s="3" t="n">
-        <v>45473.97916666666</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ds35_aedp_1000hh_sample02_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 02, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>44378</v>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>45473.97916666666</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>ds36_aedp_1000hh_sample03_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 03, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>44378</v>
-      </c>
-      <c r="F38" s="3" t="n">
-        <v>45473.97916666666</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SunDance and Fluvius aggregate datasets from North America and Belgium
- ds37/ds38: UMass Smart* SunDance hourly aggregate for 2015 (87 of 100
  sites, residential-scale and complete), with site-mean weather; CC BY 4.0
- ds39/ds40: Fluvius solar-household half-hourly aggregate for 2024 (300
  meters, Central European Time), with Open-Meteo weather at Brussels-Uccle;
  Fluvius open data licence permits redistribution with attribution
- Processing notebooks mirror the ASHD recipe and validate the exports;
  datasets registered in the download maps, metadata, docs and acknowledgements

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1955,6 +1955,178 @@
       <c r="I35" t="inlineStr">
         <is>
           <t>Generated by publication/journal_article_1/notebooks/03_acap_edp_aggregation_level/1_build_acap_edp_site_30min_checkpoints.ipynb and 2_generate_acap_edp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid ACAP-EDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ds37_sundance_hourly</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>UMass Smart* SunDance dataset, aggregate of 87 solar sites across North America</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>UMass Trace Repository (Smart* SunDance release)</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>42005</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>42369.95833333334</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>60 minute</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/00_data_exploration_and_processing/02_process_international_datasets/1_process_sundance_hourly.ipynb. Net load = use - gen per site, summed over the 87 of 100 SunDance sites that are hourly, complete and residential in scale (see sundance_site_selection.csv); sites in several North American time zones are summed on their local standard clock. CC BY 4.0; cite Chen and Irwin (2017), ACM e-Energy '17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ds38_sundance_hourly_with_weather</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ds37 enhanced with the site-mean temperature, relative humidity and wind speed from the SunDance weather files</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>UMass Trace Repository (Smart* SunDance release), public weather stations shipped with it</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>42005</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>42369.95833333334</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>60 minute</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/00_data_exploration_and_processing/02_process_international_datasets/1_process_sundance_hourly.ipynb. Net load = use - gen per site, summed over the 87 of 100 SunDance sites that are hourly, complete and residential in scale (see sundance_site_selection.csv); sites in several North American time zones are summed on their local standard clock. CC BY 4.0; cite Chen and Irwin (2017), ACM e-Energy '17. Weather is the mean over the 68 included sites that have a weather file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ds39_fluvius_pv_30min</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Fluvius digital-meter dataset, aggregate of 300 residential meters with solar panels in Flanders, Belgium</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fluvius Open Data</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>45292</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>45657.97916666666</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/00_data_exploration_and_processing/02_process_international_datasets/2_process_fluvius_pv_30min.ipynb from Fluvius open data dataset 1_50 (last updated by Fluvius 2025-09-29), profile enkel_ZP: solar panels, no heat pump, no electric vehicle. Net load = offtake - injection, summed over meters, 15-minute energy summed to 30 minutes and converted to kW; Central European Time all year. Fluvius open data licence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ds40_fluvius_pv_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ds39 enhanced with Brussels-Uccle temperature, relative humidity and wind speed from the Open-Meteo historical weather API</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Fluvius Open Data, Open-Meteo (CC BY 4.0)</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>45292</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>45657.97916666666</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/00_data_exploration_and_processing/02_process_international_datasets/2_process_fluvius_pv_30min.ipynb from Fluvius open data dataset 1_50 (last updated by Fluvius 2025-09-29), profile enkel_ZP: solar panels, no heat pump, no electric vehicle. Net load = offtake - injection, summed over meters, 15-minute energy summed to 30 minutes and converted to kW; Central European Time all year. Fluvius open data licence. Weather is hourly at 50.80 N, 4.36 E, interpolated to 30 minutes.</t>
         </is>
       </c>
     </row>

</xml_diff>